<commit_message>
remove delta_c=0.5 results from ConstrainedActionObjDoor_1c
</commit_message>
<xml_diff>
--- a/ablation_results.xlsx
+++ b/ablation_results.xlsx
@@ -4919,7 +4919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5027,58 +5027,58 @@
         <v>0.7</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>533.60 ± 464.86</t>
+          <t>398.66 ± 404.94</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0.52</v>
+        <v>0.75</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0.04 ± 0.31</t>
+          <t>0.01 ± 0.10</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>639.44 ± 418.42</t>
+          <t>688.18 ± 403.75</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.46</v>
+        <v>0.4</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>16.98 ± 20.22</t>
+          <t>19.45 ± 21.40</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>607.55 ± 456.19</t>
+          <t>392.06 ± 413.65</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>0.45</v>
+        <v>0.73</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>3.55 ± 18.65</t>
+          <t>0.02 ± 0.14</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>639.29 ± 428.22</t>
+          <t>550.21 ± 425.32</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>0.43</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>9.18 ± 14.25</t>
+          <t>11.83 ± 15.41</t>
         </is>
       </c>
     </row>
@@ -5094,282 +5094,52 @@
       <c r="E3" s="1" t="inlineStr"/>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>533.60 ± 464.86</t>
+          <t>398.66 ± 404.94</t>
         </is>
       </c>
       <c r="G3" s="1" t="n">
-        <v>0.52</v>
+        <v>0.75</v>
       </c>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t>0.04 ± 0.31</t>
+          <t>0.01 ± 0.10</t>
         </is>
       </c>
       <c r="I3" s="1" t="inlineStr">
         <is>
-          <t>639.44 ± 418.42</t>
+          <t>688.18 ± 403.75</t>
         </is>
       </c>
       <c r="J3" s="1" t="n">
-        <v>0.46</v>
+        <v>0.4</v>
       </c>
       <c r="K3" s="1" t="inlineStr">
         <is>
-          <t>16.98 ± 20.22</t>
+          <t>19.45 ± 21.40</t>
         </is>
       </c>
       <c r="L3" s="1" t="inlineStr">
         <is>
-          <t>607.55 ± 456.19</t>
+          <t>392.06 ± 413.65</t>
         </is>
       </c>
       <c r="M3" s="1" t="n">
-        <v>0.45</v>
+        <v>0.73</v>
       </c>
       <c r="N3" s="1" t="inlineStr">
         <is>
-          <t>3.55 ± 18.65</t>
+          <t>0.02 ± 0.14</t>
         </is>
       </c>
       <c r="O3" s="1" t="inlineStr">
         <is>
-          <t>639.29 ± 428.22</t>
+          <t>550.21 ± 425.32</t>
         </is>
       </c>
       <c r="P3" s="1" t="n">
-        <v>0.43</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="Q3" s="1" t="inlineStr">
-        <is>
-          <t>9.18 ± 14.25</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>--- NEW RUN: delta_g=0.7, delta_c=0.3 ---</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>Room Size</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>Num Distractor</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>Max Steps</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>Delta G</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>Delta C</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>Avg Steps C-LAMAML</t>
-        </is>
-      </c>
-      <c r="G6" s="1" t="inlineStr">
-        <is>
-          <t>Success Prob C-LAMAML</t>
-        </is>
-      </c>
-      <c r="H6" s="1" t="inlineStr">
-        <is>
-          <t>Avg Viols C-LAMAML</t>
-        </is>
-      </c>
-      <c r="I6" s="1" t="inlineStr">
-        <is>
-          <t>Avg Steps Global Only</t>
-        </is>
-      </c>
-      <c r="J6" s="1" t="inlineStr">
-        <is>
-          <t>Success Prob Global Only</t>
-        </is>
-      </c>
-      <c r="K6" s="1" t="inlineStr">
-        <is>
-          <t>Avg Viols Global Only</t>
-        </is>
-      </c>
-      <c r="L6" s="1" t="inlineStr">
-        <is>
-          <t>Avg Steps Global + Goal Adapter</t>
-        </is>
-      </c>
-      <c r="M6" s="1" t="inlineStr">
-        <is>
-          <t>Success Prob Global + Goal Adapter</t>
-        </is>
-      </c>
-      <c r="N6" s="1" t="inlineStr">
-        <is>
-          <t>Avg Viols Global + Goal Adapter</t>
-        </is>
-      </c>
-      <c r="O6" s="1" t="inlineStr">
-        <is>
-          <t>Avg Steps Global + Constraint Adapter</t>
-        </is>
-      </c>
-      <c r="P6" s="1" t="inlineStr">
-        <is>
-          <t>Success Prob Global + Constraint Adapter</t>
-        </is>
-      </c>
-      <c r="Q6" s="1" t="inlineStr">
-        <is>
-          <t>Avg Viols Global + Constraint Adapter</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>398.66 ± 404.94</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>0.01 ± 0.10</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>688.18 ± 403.75</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>19.45 ± 21.40</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>392.06 ± 413.65</t>
-        </is>
-      </c>
-      <c r="M7" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>0.02 ± 0.14</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>550.21 ± 425.32</t>
-        </is>
-      </c>
-      <c r="P7" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>11.83 ± 15.41</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>AVERAGE</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr"/>
-      <c r="C8" s="1" t="inlineStr"/>
-      <c r="D8" s="1" t="inlineStr"/>
-      <c r="E8" s="1" t="inlineStr"/>
-      <c r="F8" s="1" t="inlineStr">
-        <is>
-          <t>398.66 ± 404.94</t>
-        </is>
-      </c>
-      <c r="G8" s="1" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="H8" s="1" t="inlineStr">
-        <is>
-          <t>0.01 ± 0.10</t>
-        </is>
-      </c>
-      <c r="I8" s="1" t="inlineStr">
-        <is>
-          <t>688.18 ± 403.75</t>
-        </is>
-      </c>
-      <c r="J8" s="1" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="K8" s="1" t="inlineStr">
-        <is>
-          <t>19.45 ± 21.40</t>
-        </is>
-      </c>
-      <c r="L8" s="1" t="inlineStr">
-        <is>
-          <t>392.06 ± 413.65</t>
-        </is>
-      </c>
-      <c r="M8" s="1" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="N8" s="1" t="inlineStr">
-        <is>
-          <t>0.02 ± 0.14</t>
-        </is>
-      </c>
-      <c r="O8" s="1" t="inlineStr">
-        <is>
-          <t>550.21 ± 425.32</t>
-        </is>
-      </c>
-      <c r="P8" s="1" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="Q8" s="1" t="inlineStr">
         <is>
           <t>11.83 ± 15.41</t>
         </is>

</xml_diff>